<commit_message>
scan: seg0 2026-10-16 18:04 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-10-16.xlsx
+++ b/output/full_scan/batch_seq1_2026-10-16.xlsx
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>3.626418948861407</v>
+        <v>3.626418948861408</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>225.2905109393022</v>
+        <v>225.2905109393021</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>21.8</v>
@@ -5679,7 +5679,7 @@
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>217.7321651891394</v>
+        <v>217.7321651891393</v>
       </c>
       <c r="E99" s="2" t="n">
         <v>29.15</v>

</xml_diff>